<commit_message>
feat: add lesson for updating multiple cells using we.cell()
</commit_message>
<xml_diff>
--- a/hello_2.xlsx
+++ b/hello_2.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14.33203125" customWidth="1" min="1" max="1"/>
@@ -455,7 +455,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Johnny</t>
+          <t>John</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -557,6 +557,18 @@
       <c r="B10" t="inlineStr">
         <is>
           <t>Gray</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Neo</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Black</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add lesson for looping through spreadsheet and inserting names
</commit_message>
<xml_diff>
--- a/hello_2.xlsx
+++ b/hello_2.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14.33203125" customWidth="1" min="1" max="1"/>
@@ -560,15 +560,24 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Neo</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Black</t>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Dan</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>April</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Neal</t>
         </is>
       </c>
     </row>

</xml_diff>